<commit_message>
Update current state of the model
</commit_message>
<xml_diff>
--- a/Code/data & data_exploration/Rasmuson_dungeness_data/MegalopaeDataAndres.xlsx
+++ b/Code/data & data_exploration/Rasmuson_dungeness_data/MegalopaeDataAndres.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateoforegon-my.sharepoint.com/personal/leif_k_rasmuson_odfw_oregon_gov/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pinosa\Documents\Git\OR_trophic_model\Code\data &amp; data_exploration\Rasmuson_dungeness_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8FD0CA33-B50E-44FE-B016-469062B4426C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4CEAF93-C992-4A23-8107-11B957F004D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3AB721DC-4ACD-4C55-BF60-53565BC4C1E7}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="10300" xr2:uid="{3AB721DC-4ACD-4C55-BF60-53565BC4C1E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -414,10 +414,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFBC6D3E-028A-4B98-89AF-D029F8B243F7}">
-  <dimension ref="A1:B29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B30"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -425,7 +425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1997</v>
       </c>
@@ -433,7 +433,7 @@
         <v>1094</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1998</v>
       </c>
@@ -441,7 +441,7 @@
         <v>14900</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1999</v>
       </c>
@@ -449,7 +449,7 @@
         <v>14848</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2000</v>
       </c>
@@ -457,7 +457,7 @@
         <v>50094</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2001</v>
       </c>
@@ -465,31 +465,31 @@
         <v>61660</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2002</v>
       </c>
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2003</v>
       </c>
       <c r="B8" s="1"/>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2004</v>
       </c>
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2005</v>
       </c>
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2006</v>
       </c>
@@ -497,7 +497,7 @@
         <v>32762</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2007</v>
       </c>
@@ -505,7 +505,7 @@
         <v>1817000</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2008</v>
       </c>
@@ -513,7 +513,7 @@
         <v>1770000</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>2009</v>
       </c>
@@ -521,7 +521,7 @@
         <v>2398833</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>2010</v>
       </c>
@@ -529,7 +529,7 @@
         <v>912011</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>2011</v>
       </c>
@@ -537,7 +537,7 @@
         <v>162181</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2012</v>
       </c>
@@ -545,7 +545,7 @@
         <v>288403</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2013</v>
       </c>
@@ -553,7 +553,7 @@
         <v>2290868</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>2014</v>
       </c>
@@ -561,7 +561,7 @@
         <v>197242</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>2015</v>
       </c>
@@ -569,7 +569,7 @@
         <v>43652</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>2016</v>
       </c>
@@ -577,7 +577,7 @@
         <v>3105</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2017</v>
       </c>
@@ -585,7 +585,7 @@
         <v>117359</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2018</v>
       </c>
@@ -593,7 +593,7 @@
         <v>2795426</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2019</v>
       </c>
@@ -601,7 +601,7 @@
         <v>425823</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2020</v>
       </c>
@@ -609,7 +609,7 @@
         <v>161062</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2021</v>
       </c>
@@ -617,7 +617,7 @@
         <v>188728</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2022</v>
       </c>
@@ -625,7 +625,7 @@
         <v>63079</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>2023</v>
       </c>
@@ -633,12 +633,18 @@
         <v>2472277</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>2024</v>
       </c>
       <c r="B29" s="1">
         <v>6141</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B30" s="1">
+        <f>AVERAGE(B2:B29)</f>
+        <v>678689.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>